<commit_message>
fix(pdf): overhaul absence inquiry form 20 with fixed table layout, 3-column header, and high-res canvas scaling
</commit_message>
<xml_diff>
--- a/منسوبات ث5.xlsx
+++ b/منسوبات ث5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seham\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mo0od\Desktop\منصة الغياب الإدارية 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5DB7DDB-A9BB-4256-9F51-FCAA1A726FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F18643-5E9A-439E-977D-179C1BD718AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -480,7 +480,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -512,10 +512,20 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="ارتباط تشعبي" xfId="1" builtinId="8"/>
-    <cellStyle name="عادي" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -864,7 +874,7 @@
   <cols>
     <col min="1" max="1" width="11.796875" customWidth="1"/>
     <col min="2" max="2" width="13.69921875" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="3" max="3" width="33.796875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -874,7 +884,7 @@
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
@@ -890,14 +900,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="19.2">
+    <row r="2" spans="1:7">
       <c r="A2" s="5">
         <v>1010669594</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="11">
         <v>966509683264</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -913,14 +923,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="19.2">
+    <row r="3" spans="1:7">
       <c r="A3" s="5">
         <v>1043325131</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="11">
         <v>966550801116</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -936,14 +946,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="19.2">
+    <row r="4" spans="1:7">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="11">
         <v>966502563997</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -959,14 +969,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="19.2">
+    <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="11">
         <v>966552523681</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -982,14 +992,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="19.2">
+    <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="11">
         <v>966531193174</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -1005,14 +1015,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="19.2">
+    <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="11">
         <v>966552832729</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -1028,14 +1038,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="19.2">
+    <row r="8" spans="1:7">
       <c r="A8" s="5">
         <v>1065712158</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="11">
         <v>966556971084</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1051,14 +1061,14 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="19.2">
+    <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="11">
         <v>966557416665</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -1074,14 +1084,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="19.2">
+    <row r="10" spans="1:7">
       <c r="A10" s="5">
         <v>1038667364</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="11">
         <v>966554546789</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1104,7 +1114,7 @@
       <c r="B11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="11">
         <v>966500046770</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -1120,14 +1130,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="19.2">
+    <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="11">
         <v>966552244081</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1143,14 +1153,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="19.2">
+    <row r="13" spans="1:7">
       <c r="A13" s="5">
         <v>1027408390</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="11">
         <v>966540522692</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1173,7 +1183,7 @@
       <c r="B14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="11">
         <v>966538544464</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1189,14 +1199,14 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="19.2">
+    <row r="15" spans="1:7">
       <c r="A15" s="5">
         <v>1035114642</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="11">
         <v>966533926716</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1212,14 +1222,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="19.2">
+    <row r="16" spans="1:7">
       <c r="A16" s="5">
         <v>1021326572</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="11">
         <v>966555749516</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -1235,14 +1245,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="19.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="11">
         <v>966569418491</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1265,7 +1275,7 @@
       <c r="B18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="11">
         <v>966540773232</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -1281,14 +1291,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="19.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="5">
         <v>1029416573</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="11">
         <v>966559134228</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -1304,14 +1314,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="19.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="5">
         <v>1060106364</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="11">
         <v>966567756734</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1334,7 +1344,7 @@
       <c r="B21" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="11">
         <v>966500581322</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -1357,7 +1367,7 @@
       <c r="B22" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="11">
         <v>966504501406</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1373,14 +1383,14 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="19.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="11">
         <v>966531031064</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1396,14 +1406,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="19.2">
+    <row r="24" spans="1:7">
       <c r="A24" s="5">
         <v>1018584357</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" s="11">
         <v>966580127127</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1419,14 +1429,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="19.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="5">
         <v>1071632648</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="11">
         <v>966560342997</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1442,14 +1452,14 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="19.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="11">
         <v>966500570822</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1472,7 +1482,7 @@
       <c r="B27" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="11">
         <v>966555057874</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -1488,14 +1498,14 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="19.2">
+    <row r="28" spans="1:7">
       <c r="A28" s="5" t="s">
         <v>66</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="1">
+      <c r="C28" s="11">
         <v>966550220808</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1511,14 +1521,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="19.2">
+    <row r="29" spans="1:7">
       <c r="A29" s="5" t="s">
         <v>68</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="11">
         <v>966560376050</v>
       </c>
       <c r="D29" s="1" t="s">
@@ -1534,14 +1544,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="19.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="11">
         <v>966501341969</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -1557,14 +1567,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="19.2">
+    <row r="31" spans="1:7">
       <c r="A31" s="5">
         <v>1016978650</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="11">
         <v>966550074422</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -1580,14 +1590,14 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="19.2">
+    <row r="32" spans="1:7">
       <c r="A32" s="5">
         <v>1073463562</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="11">
         <v>966532656942</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1603,14 +1613,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="19.2">
+    <row r="33" spans="1:7">
       <c r="A33" s="5">
         <v>1008480368</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="11">
         <v>966504520578</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1626,14 +1636,14 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="19.2">
+    <row r="34" spans="1:7">
       <c r="A34" s="5" t="s">
         <v>75</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="11">
         <v>966508727560</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -1649,14 +1659,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="19.2">
+    <row r="35" spans="1:7">
       <c r="A35" s="5">
         <v>1012793475</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="11">
         <v>966564954507</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1672,14 +1682,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="19.2">
+    <row r="36" spans="1:7">
       <c r="A36" s="5">
         <v>1032930222</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" s="11">
         <v>966540444543</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1702,7 +1712,7 @@
       <c r="B37" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" s="11">
         <v>966506536278</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -1718,14 +1728,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="19.2">
+    <row r="38" spans="1:7">
       <c r="A38" s="7">
         <v>1015524257</v>
       </c>
       <c r="B38" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="13">
         <v>966556536776</v>
       </c>
       <c r="D38" s="8" t="s">
@@ -1755,6 +1765,7 @@
     <hyperlink ref="G1" r:id="rId7" display="javascript:__doPostBack('ctl00$PlaceHolderMain$gvUserInfo','Sort$MajorDesc')" xr:uid="{DD3E82C8-017A-4C38-9772-507CEEFBDCA6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>